<commit_message>
replace with 26-04-2026 update
</commit_message>
<xml_diff>
--- a/SPER and HCP_R&P streamlit dash.xlsx
+++ b/SPER and HCP_R&P streamlit dash.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wfp.sharepoint.com/sites/MozambiqueCOBeneficiaryData-Activity4/Shared Documents/Activity 4 - Social Protection/Mozambique_HCP e SPER/Dashboard_SPER HCP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="953" documentId="11_B941838DCB70CED39E8AF10BAAC34C2D2E3290C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73164FB4-E2D8-475B-B141-72AEA6EB7F14}"/>
+  <xr:revisionPtr revIDLastSave="959" documentId="11_B941838DCB70CED39E8AF10BAAC34C2D2E3290C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92C9D94E-5DCB-49A0-A399-7BF1A68F3BC0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="104">
   <si>
     <t xml:space="preserve">Beneficiários pagos </t>
   </si>
@@ -313,9 +313,6 @@
   </si>
   <si>
     <t>Registos  nao iniciados</t>
-  </si>
-  <si>
-    <t>Pagamento realizado</t>
   </si>
   <si>
     <t>Analise de dados em curso</t>
@@ -967,40 +964,40 @@
   <sheetData>
     <row r="1" spans="2:23" s="44" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="B1" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="D1" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="E1" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="37" t="s">
+      <c r="F1" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="G1" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="G1" s="37" t="s">
+      <c r="H1" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="I1" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="J1" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="H1" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="I1" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="J1" s="26" t="s">
+      <c r="K1" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="L1" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="M1" s="47" t="s">
         <v>99</v>
-      </c>
-      <c r="K1" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="L1" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="M1" s="47" t="s">
-        <v>100</v>
       </c>
       <c r="N1" s="39" t="s">
         <v>0</v>
@@ -1149,7 +1146,7 @@
       <c r="T3" s="2"/>
       <c r="U3" s="5"/>
       <c r="V3" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W3" s="5"/>
     </row>
@@ -1323,7 +1320,7 @@
       <c r="U6" s="29">
         <v>13</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="5" t="s">
         <v>89</v>
       </c>
       <c r="W6" s="20"/>
@@ -1384,7 +1381,7 @@
       <c r="U7" s="29">
         <v>40</v>
       </c>
-      <c r="V7" s="29" t="s">
+      <c r="V7" s="5" t="s">
         <v>89</v>
       </c>
       <c r="W7" s="20"/>
@@ -1503,7 +1500,7 @@
         <v>127</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="W9" s="5"/>
     </row>
@@ -1619,7 +1616,7 @@
         <v>86</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="W11" s="5"/>
     </row>
@@ -2448,7 +2445,7 @@
       <c r="T26" s="5"/>
       <c r="U26" s="5"/>
       <c r="V26" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W26" s="5"/>
     </row>
@@ -2672,7 +2669,7 @@
       <c r="T30" s="5"/>
       <c r="U30" s="5"/>
       <c r="V30" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W30" s="5"/>
     </row>
@@ -2731,7 +2728,7 @@
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
       <c r="V31" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W31" s="5"/>
     </row>
@@ -2790,7 +2787,7 @@
       <c r="T32" s="5"/>
       <c r="U32" s="5"/>
       <c r="V32" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W32" s="5"/>
     </row>
@@ -2904,7 +2901,7 @@
       <c r="T34" s="5"/>
       <c r="U34" s="5"/>
       <c r="V34" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W34" s="5"/>
     </row>
@@ -3128,7 +3125,7 @@
       <c r="T38" s="5"/>
       <c r="U38" s="5"/>
       <c r="V38" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W38" s="5"/>
     </row>
@@ -3242,7 +3239,7 @@
       <c r="T40" s="5"/>
       <c r="U40" s="5"/>
       <c r="V40" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W40" s="5"/>
     </row>
@@ -4730,7 +4727,7 @@
       <c r="T67" s="5"/>
       <c r="U67" s="5"/>
       <c r="V67" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W67" s="5"/>
     </row>
@@ -4789,7 +4786,7 @@
       <c r="T68" s="5"/>
       <c r="U68" s="5"/>
       <c r="V68" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W68" s="5"/>
     </row>
@@ -4848,7 +4845,7 @@
       <c r="T69" s="5"/>
       <c r="U69" s="5"/>
       <c r="V69" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W69" s="5"/>
     </row>
@@ -4962,7 +4959,7 @@
       <c r="T71" s="5"/>
       <c r="U71" s="5"/>
       <c r="V71" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W71" s="5"/>
     </row>
@@ -5021,7 +5018,7 @@
       <c r="T72" s="5"/>
       <c r="U72" s="5"/>
       <c r="V72" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W72" s="5"/>
     </row>
@@ -5080,7 +5077,7 @@
       <c r="T73" s="5"/>
       <c r="U73" s="5"/>
       <c r="V73" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W73" s="5"/>
     </row>
@@ -5194,7 +5191,7 @@
       <c r="T75" s="5"/>
       <c r="U75" s="5"/>
       <c r="V75" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W75" s="5"/>
     </row>
@@ -5473,7 +5470,7 @@
       <c r="T80" s="5"/>
       <c r="U80" s="5"/>
       <c r="V80" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W80" s="5"/>
     </row>
@@ -5532,7 +5529,7 @@
       <c r="T81" s="5"/>
       <c r="U81" s="5"/>
       <c r="V81" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W81" s="5"/>
     </row>
@@ -5592,7 +5589,7 @@
       <c r="U82" s="29">
         <v>4</v>
       </c>
-      <c r="V82" s="29" t="s">
+      <c r="V82" s="5" t="s">
         <v>89</v>
       </c>
       <c r="W82" s="5"/>
@@ -5762,7 +5759,7 @@
       <c r="T85" s="5"/>
       <c r="U85" s="5"/>
       <c r="V85" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W85" s="5"/>
     </row>
@@ -6536,7 +6533,7 @@
       <c r="T99" s="5"/>
       <c r="U99" s="5"/>
       <c r="V99" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W99" s="5"/>
     </row>
@@ -6595,7 +6592,7 @@
       <c r="T100" s="5"/>
       <c r="U100" s="5"/>
       <c r="V100" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W100" s="5"/>
     </row>
@@ -6652,12 +6649,9 @@
         <v>-8</v>
       </c>
       <c r="T101" s="5"/>
-      <c r="U101" s="29" t="e">
-        <f>J101-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="U101" s="29"/>
       <c r="V101" s="29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="W101" s="5"/>
     </row>
@@ -6771,7 +6765,7 @@
       <c r="T103" s="5"/>
       <c r="U103" s="5"/>
       <c r="V103" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W103" s="5"/>
     </row>
@@ -6830,7 +6824,7 @@
       <c r="T104" s="5"/>
       <c r="U104" s="5"/>
       <c r="V104" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W104" s="5"/>
     </row>
@@ -6889,7 +6883,7 @@
       <c r="T105" s="5"/>
       <c r="U105" s="5"/>
       <c r="V105" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W105" s="5"/>
     </row>
@@ -7005,7 +6999,7 @@
         <f>705-J107</f>
         <v>-589</v>
       </c>
-      <c r="V107" s="29" t="s">
+      <c r="V107" s="5" t="s">
         <v>89</v>
       </c>
       <c r="W107" s="5"/>
@@ -7419,16 +7413,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="13b3eab5-f992-450e-ab7b-a05d8005a6f7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100264EC166BFEF9644B5A7611DE06D4E97" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="95cdffe3b25d1c8c303cf4abe9ec6caf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="13b3eab5-f992-450e-ab7b-a05d8005a6f7" xmlns:ns3="967e33a3-a708-417c-8aeb-92451b8d7f34" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="006918caa63e88534e48a2eb234fbabf" ns2:_="" ns3:_="">
     <xsd:import namespace="13b3eab5-f992-450e-ab7b-a05d8005a6f7"/>
@@ -7639,6 +7623,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="13b3eab5-f992-450e-ab7b-a05d8005a6f7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{005C5C98-AA8F-4EAD-974E-073E947FF7E2}">
   <ds:schemaRefs>
@@ -7648,16 +7642,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECC8EB4F-E3F4-402D-BE00-3B0AFBB3276C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="13b3eab5-f992-450e-ab7b-a05d8005a6f7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{010C1924-A215-4D87-A9B4-1E5E1CCDF1FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7674,4 +7658,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECC8EB4F-E3F4-402D-BE00-3B0AFBB3276C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="13b3eab5-f992-450e-ab7b-a05d8005a6f7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update the data to include registration out of network
</commit_message>
<xml_diff>
--- a/SPER and HCP_R&P streamlit dash.xlsx
+++ b/SPER and HCP_R&P streamlit dash.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wfp.sharepoint.com/sites/MozambiqueCOBeneficiaryData-Activity4/Shared Documents/Activity 4 - Social Protection/Mozambique_HCP e SPER/Dashboard_SPER HCP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="959" documentId="11_B941838DCB70CED39E8AF10BAAC34C2D2E3290C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92C9D94E-5DCB-49A0-A399-7BF1A68F3BC0}"/>
+  <xr:revisionPtr revIDLastSave="965" documentId="11_B941838DCB70CED39E8AF10BAAC34C2D2E3290C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA5C1A35-C967-4A9B-8605-CEA022721D24}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1178,11 +1178,11 @@
         <v>339</v>
       </c>
       <c r="K4" s="23">
-        <v>70</v>
+        <v>339</v>
       </c>
       <c r="L4" s="51">
         <f t="shared" si="1"/>
-        <v>69.329896907216494</v>
+        <v>0</v>
       </c>
       <c r="M4" s="50">
         <f t="shared" si="2"/>
@@ -1200,7 +1200,7 @@
       <c r="R4" s="3"/>
       <c r="S4" s="22">
         <f t="shared" si="4"/>
-        <v>-269</v>
+        <v>0</v>
       </c>
       <c r="T4" s="3"/>
       <c r="U4" s="5"/>
@@ -1588,7 +1588,9 @@
       <c r="J11" s="13">
         <v>141</v>
       </c>
-      <c r="K11" s="28"/>
+      <c r="K11" s="28">
+        <v>53</v>
+      </c>
       <c r="L11" s="51">
         <f t="shared" si="1"/>
         <v>15.807174887892378</v>
@@ -1609,7 +1611,7 @@
       <c r="R11" s="5"/>
       <c r="S11" s="22">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="5">
@@ -4701,10 +4703,12 @@
       <c r="J67" s="15">
         <v>928</v>
       </c>
-      <c r="K67" s="24"/>
+      <c r="K67" s="24">
+        <v>193</v>
+      </c>
       <c r="L67" s="51">
         <f t="shared" ref="L67:L114" si="6">(MAX(I67,(J67-K67))/E67)*100</f>
-        <v>36.913285600636435</v>
+        <v>30.469371519490849</v>
       </c>
       <c r="M67" s="50">
         <f t="shared" ref="M67:M114" si="7">(H67/E67)*100</f>
@@ -4722,7 +4726,7 @@
       <c r="R67" s="5"/>
       <c r="S67" s="22">
         <f t="shared" ref="S67:S114" si="9">I67-(J67-K67)</f>
-        <v>-162</v>
+        <v>31</v>
       </c>
       <c r="T67" s="5"/>
       <c r="U67" s="5"/>
@@ -4819,10 +4823,12 @@
       <c r="J69" s="31">
         <v>464</v>
       </c>
-      <c r="K69" s="24"/>
+      <c r="K69" s="24">
+        <v>307</v>
+      </c>
       <c r="L69" s="51">
         <f t="shared" si="6"/>
-        <v>59.487179487179489</v>
+        <v>26.666666666666668</v>
       </c>
       <c r="M69" s="50">
         <f t="shared" si="7"/>
@@ -4840,7 +4846,7 @@
       <c r="R69" s="5"/>
       <c r="S69" s="22">
         <f t="shared" si="9"/>
-        <v>-256</v>
+        <v>51</v>
       </c>
       <c r="T69" s="5"/>
       <c r="U69" s="5"/>
@@ -4933,10 +4939,12 @@
       <c r="J71" s="32">
         <v>1786</v>
       </c>
-      <c r="K71" s="24"/>
+      <c r="K71" s="24">
+        <v>786</v>
+      </c>
       <c r="L71" s="51">
         <f t="shared" si="6"/>
-        <v>91.542798564838549</v>
+        <v>51.255766273705795</v>
       </c>
       <c r="M71" s="50">
         <f t="shared" si="7"/>
@@ -4954,7 +4962,7 @@
       <c r="R71" s="5"/>
       <c r="S71" s="22">
         <f t="shared" si="9"/>
-        <v>-786</v>
+        <v>0</v>
       </c>
       <c r="T71" s="5"/>
       <c r="U71" s="5"/>
@@ -5165,10 +5173,12 @@
       <c r="J75" s="31">
         <v>993</v>
       </c>
-      <c r="K75" s="24"/>
+      <c r="K75" s="24">
+        <v>45</v>
+      </c>
       <c r="L75" s="51">
         <f t="shared" si="6"/>
-        <v>90.519598906107575</v>
+        <v>86.417502278942564</v>
       </c>
       <c r="M75" s="50">
         <f t="shared" si="7"/>
@@ -5186,7 +5196,7 @@
       <c r="R75" s="5"/>
       <c r="S75" s="22">
         <f t="shared" si="9"/>
-        <v>-45</v>
+        <v>0</v>
       </c>
       <c r="T75" s="5"/>
       <c r="U75" s="5"/>
@@ -7404,12 +7414,13 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="13b3eab5-f992-450e-ab7b-a05d8005a6f7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7624,19 +7635,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="13b3eab5-f992-450e-ab7b-a05d8005a6f7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{005C5C98-AA8F-4EAD-974E-073E947FF7E2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECC8EB4F-E3F4-402D-BE00-3B0AFBB3276C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="13b3eab5-f992-450e-ab7b-a05d8005a6f7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7661,11 +7673,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECC8EB4F-E3F4-402D-BE00-3B0AFBB3276C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{005C5C98-AA8F-4EAD-974E-073E947FF7E2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="13b3eab5-f992-450e-ab7b-a05d8005a6f7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>